<commit_message>
성형 스케줄링 제약조건 7건 추가/개정 (PDD-02 v1.1, PDD-04 v1.4, SRS v1.4)
- BR-V07 정책 전환: 앵글 교체 최소화 → 당일 락 + 일말 일괄 교체
- BR-V12~V17 신규: capa 분기(우선순위/KD), 28422-08HA0 LP-01 단일,
  28422-2M800 우측·≤2, 28421-2M800 좌측·≤2, 규격<7 가류기당 ≤4
- 성형 마스터에 K(좌측셋팅)/L(우측셋팅) 컬럼 신설, 압출 B(규격) cross-reference
- BR-V12/V13은 수주정보 통합 작업 완료 후 활성

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phase 1/2.Raw Materials/Vulcanization/성형공정_제약조건.xlsx
+++ b/Phase 1/2.Raw Materials/Vulcanization/성형공정_제약조건.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="현재_통합_문서" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SWI\통합계획\클로드\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Antigavity Workspace\Internal Production Scheduling Project\Phase 1\2.Raw Materials\Vulcanization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B49AFAE-DF57-4D5D-89AD-6D7CD24B8DEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCC7E029-2651-4061-B2F1-0D79E38223C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F2A8E265-CF04-4D2D-B7BD-04B0FE4810B2}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="95">
   <si>
     <t>HOSE</t>
   </si>
@@ -359,6 +359,14 @@
   </si>
   <si>
     <t>\</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>좌측셋팅</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>우측셋팅</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -854,16 +862,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{790A88E3-97BA-4B56-9AAE-0A981A51B651}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A2:T48"/>
+  <dimension ref="A2:V48"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="13.625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9" style="4"/>
-    <col min="18" max="18" width="33.875" style="5" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9" style="4"/>
+    <col min="20" max="20" width="33.875" style="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:18">
+    <row r="2" spans="1:20">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -894,29 +902,35 @@
       <c r="J2" s="2">
         <v>4</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="M2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="M2" s="3">
-        <v>1</v>
-      </c>
-      <c r="N2" s="3">
+      <c r="O2" s="3">
+        <v>1</v>
+      </c>
+      <c r="P2" s="3">
         <v>2</v>
       </c>
-      <c r="O2" s="3">
+      <c r="Q2" s="3">
         <v>3</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="S2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="R2" s="5" t="s">
+      <c r="T2" s="5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:18">
+    <row r="3" spans="1:20">
       <c r="A3" s="6" t="s">
         <v>10</v>
       </c>
@@ -947,29 +961,35 @@
       <c r="J3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="6">
-        <v>20</v>
-      </c>
-      <c r="L3" s="6">
-        <v>1</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="N3" s="6" t="s">
-        <v>12</v>
+      <c r="K3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M3" s="6">
+        <v>20</v>
+      </c>
+      <c r="N3" s="6">
+        <v>1</v>
       </c>
       <c r="O3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="Q3" s="7" t="s">
+      <c r="P3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="S3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="R3" s="8" t="s">
+      <c r="T3" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:18">
+    <row r="4" spans="1:20">
       <c r="A4" s="6" t="s">
         <v>15</v>
       </c>
@@ -1000,29 +1020,35 @@
       <c r="J4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K4" s="6">
-        <v>20</v>
-      </c>
-      <c r="L4" s="6">
-        <v>1</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="N4" s="6" t="s">
-        <v>12</v>
+      <c r="K4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M4" s="6">
+        <v>20</v>
+      </c>
+      <c r="N4" s="6">
+        <v>1</v>
       </c>
       <c r="O4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="Q4" s="4" t="s">
+      <c r="P4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="S4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="R4" s="8" t="s">
+      <c r="T4" s="8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:18">
+    <row r="5" spans="1:20">
       <c r="A5" s="9" t="s">
         <v>18</v>
       </c>
@@ -1053,29 +1079,35 @@
       <c r="J5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K5" s="6">
-        <v>20</v>
-      </c>
-      <c r="L5" s="6">
-        <v>1</v>
-      </c>
-      <c r="M5" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="N5" s="6" t="s">
-        <v>12</v>
+      <c r="K5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M5" s="6">
+        <v>20</v>
+      </c>
+      <c r="N5" s="6">
+        <v>1</v>
       </c>
       <c r="O5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="Q5" s="7" t="s">
+      <c r="P5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="S5" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="R5" s="8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18">
+      <c r="T5" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20">
       <c r="A6" s="9" t="s">
         <v>21</v>
       </c>
@@ -1106,29 +1138,35 @@
       <c r="J6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K6" s="6">
-        <v>20</v>
-      </c>
-      <c r="L6" s="6">
-        <v>1</v>
-      </c>
-      <c r="M6" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="N6" s="6" t="s">
-        <v>12</v>
+      <c r="K6" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M6" s="6">
+        <v>20</v>
+      </c>
+      <c r="N6" s="6">
+        <v>1</v>
       </c>
       <c r="O6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="Q6" s="4" t="s">
+      <c r="P6" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q6" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="S6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="R6" s="5" t="s">
+      <c r="T6" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:18">
+    <row r="7" spans="1:20">
       <c r="A7" s="9" t="s">
         <v>24</v>
       </c>
@@ -1157,29 +1195,35 @@
       <c r="J7" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K7" s="6">
-        <v>20</v>
-      </c>
-      <c r="L7" s="6">
-        <v>1</v>
-      </c>
-      <c r="M7" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="N7" s="6" t="s">
-        <v>12</v>
+      <c r="K7" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M7" s="6">
+        <v>20</v>
+      </c>
+      <c r="N7" s="6">
+        <v>1</v>
       </c>
       <c r="O7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="Q7" s="7" t="s">
+      <c r="P7" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q7" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="S7" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="R7" s="8" t="s">
+      <c r="T7" s="8" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:18">
+    <row r="8" spans="1:20">
       <c r="A8" s="6" t="s">
         <v>27</v>
       </c>
@@ -1210,29 +1254,35 @@
       <c r="J8" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="6">
-        <v>20</v>
-      </c>
-      <c r="L8" s="6">
-        <v>1</v>
-      </c>
-      <c r="M8" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="N8" s="6" t="s">
-        <v>12</v>
+      <c r="K8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M8" s="6">
+        <v>20</v>
+      </c>
+      <c r="N8" s="6">
+        <v>1</v>
       </c>
       <c r="O8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="Q8" s="4" t="s">
+      <c r="P8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="S8" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="R8" s="5" t="s">
+      <c r="T8" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:18">
+    <row r="9" spans="1:20">
       <c r="A9" s="6" t="s">
         <v>30</v>
       </c>
@@ -1263,29 +1313,35 @@
       <c r="J9" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K9" s="6">
-        <v>20</v>
-      </c>
-      <c r="L9" s="6">
-        <v>1</v>
-      </c>
-      <c r="M9" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="N9" s="6" t="s">
-        <v>12</v>
+      <c r="K9" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M9" s="6">
+        <v>20</v>
+      </c>
+      <c r="N9" s="6">
+        <v>1</v>
       </c>
       <c r="O9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="Q9" s="7" t="s">
+      <c r="P9" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q9" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="S9" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="R9" s="5" t="s">
+      <c r="T9" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:18">
+    <row r="10" spans="1:20">
       <c r="A10" s="9" t="s">
         <v>33</v>
       </c>
@@ -1316,29 +1372,35 @@
       <c r="J10" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K10" s="6">
-        <v>20</v>
-      </c>
-      <c r="L10" s="6">
-        <v>1</v>
-      </c>
-      <c r="M10" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="N10" s="6" t="s">
-        <v>12</v>
+      <c r="K10" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L10" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M10" s="6">
+        <v>20</v>
+      </c>
+      <c r="N10" s="6">
+        <v>1</v>
       </c>
       <c r="O10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="Q10" s="4" t="s">
+      <c r="P10" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q10" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="S10" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="R10" s="5" t="s">
+      <c r="T10" s="5" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:18">
+    <row r="11" spans="1:20">
       <c r="A11" s="6" t="s">
         <v>36</v>
       </c>
@@ -1369,27 +1431,33 @@
       <c r="J11" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="K11" s="6">
+      <c r="K11" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M11" s="6">
         <v>0</v>
       </c>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="N11" s="6" t="s">
-        <v>11</v>
-      </c>
+      <c r="N11" s="6"/>
       <c r="O11" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="Q11" s="7" t="s">
+      <c r="P11" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q11" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="S11" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="R11" s="5" t="s">
+      <c r="T11" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:18">
+    <row r="12" spans="1:20">
       <c r="A12" s="6" t="s">
         <v>39</v>
       </c>
@@ -1418,29 +1486,35 @@
       <c r="J12" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K12" s="6">
-        <v>20</v>
-      </c>
-      <c r="L12" s="6">
-        <v>1</v>
-      </c>
-      <c r="M12" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="N12" s="6" t="s">
-        <v>12</v>
+      <c r="K12" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L12" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M12" s="6">
+        <v>20</v>
+      </c>
+      <c r="N12" s="6">
+        <v>1</v>
       </c>
       <c r="O12" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="Q12" s="4" t="s">
+      <c r="P12" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q12" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="S12" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="R12" s="5" t="s">
+      <c r="T12" s="5" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:18">
+    <row r="13" spans="1:20">
       <c r="A13" s="6" t="s">
         <v>42</v>
       </c>
@@ -1471,27 +1545,33 @@
       <c r="J13" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="K13" s="6">
+      <c r="K13" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L13" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M13" s="6">
         <v>0</v>
       </c>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="N13" s="6" t="s">
-        <v>11</v>
-      </c>
+      <c r="N13" s="6"/>
       <c r="O13" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="Q13" s="7" t="s">
+      <c r="P13" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q13" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="S13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="R13" s="5" t="s">
+      <c r="T13" s="5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:18">
+    <row r="14" spans="1:20">
       <c r="A14" s="6" t="s">
         <v>45</v>
       </c>
@@ -1522,29 +1602,35 @@
       <c r="J14" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K14" s="6">
-        <v>20</v>
-      </c>
-      <c r="L14" s="6">
-        <v>1</v>
-      </c>
-      <c r="M14" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="N14" s="6" t="s">
-        <v>12</v>
+      <c r="K14" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L14" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M14" s="6">
+        <v>20</v>
+      </c>
+      <c r="N14" s="6">
+        <v>1</v>
       </c>
       <c r="O14" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="Q14" s="4" t="s">
+      <c r="P14" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q14" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="S14" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="R14" s="5" t="s">
+      <c r="T14" s="5" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:18">
+    <row r="15" spans="1:20">
       <c r="A15" s="6" t="s">
         <v>48</v>
       </c>
@@ -1575,29 +1661,35 @@
       <c r="J15" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K15" s="6">
-        <v>20</v>
-      </c>
-      <c r="L15" s="6">
-        <v>1</v>
-      </c>
-      <c r="M15" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="N15" s="6" t="s">
-        <v>12</v>
+      <c r="K15" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M15" s="6">
+        <v>20</v>
+      </c>
+      <c r="N15" s="6">
+        <v>1</v>
       </c>
       <c r="O15" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="Q15" s="7" t="s">
+      <c r="P15" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q15" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="S15" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="R15" s="5" t="s">
+      <c r="T15" s="5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:18">
+    <row r="16" spans="1:20">
       <c r="A16" s="6" t="s">
         <v>51</v>
       </c>
@@ -1628,29 +1720,35 @@
       <c r="J16" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K16" s="6">
-        <v>20</v>
-      </c>
-      <c r="L16" s="6">
-        <v>1</v>
-      </c>
-      <c r="M16" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="N16" s="6" t="s">
-        <v>12</v>
+      <c r="K16" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L16" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M16" s="6">
+        <v>20</v>
+      </c>
+      <c r="N16" s="6">
+        <v>1</v>
       </c>
       <c r="O16" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="Q16" s="4" t="s">
+      <c r="P16" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q16" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="S16" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="R16" s="5" t="s">
+      <c r="T16" s="5" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="17" spans="1:20">
+    <row r="17" spans="1:22">
       <c r="A17" s="6" t="s">
         <v>54</v>
       </c>
@@ -1681,24 +1779,30 @@
       <c r="J17" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="K17" s="6">
+      <c r="K17" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L17" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M17" s="6">
         <v>0</v>
       </c>
-      <c r="L17" s="6">
-        <v>1</v>
-      </c>
-      <c r="M17" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="N17" s="6" t="s">
-        <v>11</v>
+      <c r="N17" s="6">
+        <v>1</v>
       </c>
       <c r="O17" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="Q17" s="7"/>
-    </row>
-    <row r="18" spans="1:20">
+      <c r="P17" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q17" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="S17" s="7"/>
+    </row>
+    <row r="18" spans="1:22">
       <c r="A18" s="6" t="s">
         <v>55</v>
       </c>
@@ -1727,23 +1831,29 @@
       <c r="J18" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K18" s="6">
-        <v>20</v>
-      </c>
-      <c r="L18" s="6">
-        <v>1</v>
-      </c>
-      <c r="M18" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="N18" s="10" t="s">
-        <v>11</v>
+      <c r="K18" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M18" s="6">
+        <v>20</v>
+      </c>
+      <c r="N18" s="6">
+        <v>1</v>
       </c>
       <c r="O18" s="10" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="19" spans="1:20">
+        <v>11</v>
+      </c>
+      <c r="P18" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q18" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22">
       <c r="A19" s="6" t="s">
         <v>56</v>
       </c>
@@ -1774,30 +1884,36 @@
       <c r="J19" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K19" s="6">
-        <v>20</v>
-      </c>
-      <c r="L19" s="6">
-        <v>1</v>
-      </c>
-      <c r="M19" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="N19" s="10" t="s">
-        <v>12</v>
+      <c r="K19" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L19" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M19" s="6">
+        <v>20</v>
+      </c>
+      <c r="N19" s="6">
+        <v>1</v>
       </c>
       <c r="O19" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="Q19" s="7"/>
-      <c r="R19" s="5" t="s">
+      <c r="P19" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q19" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="S19" s="7"/>
+      <c r="T19" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="S19">
+      <c r="U19">
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:20">
+    <row r="20" spans="1:22">
       <c r="A20" s="6" t="s">
         <v>58</v>
       </c>
@@ -1828,29 +1944,35 @@
       <c r="J20" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="K20" s="6">
-        <v>20</v>
-      </c>
-      <c r="L20" s="6">
-        <v>1</v>
-      </c>
-      <c r="M20" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N20" s="10" t="s">
-        <v>12</v>
+      <c r="K20" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L20" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M20" s="6">
+        <v>20</v>
+      </c>
+      <c r="N20" s="6">
+        <v>1</v>
       </c>
       <c r="O20" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="R20" s="5" t="s">
+      <c r="P20" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q20" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="T20" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="S20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:20">
+      <c r="U20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22">
       <c r="A21" s="6" t="s">
         <v>60</v>
       </c>
@@ -1879,21 +2001,27 @@
       <c r="J21" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K21" s="6">
+      <c r="K21" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L21" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M21" s="6">
         <v>0</v>
       </c>
-      <c r="L21" s="6"/>
-      <c r="M21" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="N21" s="6" t="s">
-        <v>11</v>
-      </c>
+      <c r="N21" s="6"/>
       <c r="O21" s="6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="22" spans="1:20">
+      <c r="P21" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q21" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22">
       <c r="A22" s="6" t="s">
         <v>61</v>
       </c>
@@ -1924,21 +2052,27 @@
       <c r="J22" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="K22" s="6">
+      <c r="K22" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L22" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M22" s="6">
         <v>0</v>
       </c>
-      <c r="L22" s="6"/>
-      <c r="M22" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="N22" s="6" t="s">
-        <v>11</v>
-      </c>
+      <c r="N22" s="6"/>
       <c r="O22" s="6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="23" spans="1:20">
+      <c r="P22" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q22" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22">
       <c r="A23" s="6" t="s">
         <v>62</v>
       </c>
@@ -1969,23 +2103,29 @@
       <c r="J23" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K23" s="6">
-        <v>20</v>
-      </c>
-      <c r="L23" s="6">
-        <v>1</v>
-      </c>
-      <c r="M23" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N23" s="10" t="s">
-        <v>12</v>
+      <c r="K23" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L23" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M23" s="6">
+        <v>20</v>
+      </c>
+      <c r="N23" s="6">
+        <v>1</v>
       </c>
       <c r="O23" s="10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="24" spans="1:20">
+        <v>12</v>
+      </c>
+      <c r="P23" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q23" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22">
       <c r="A24" s="6" t="s">
         <v>63</v>
       </c>
@@ -2014,23 +2154,29 @@
       <c r="J24" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K24" s="6">
-        <v>20</v>
-      </c>
-      <c r="L24" s="6">
-        <v>1</v>
-      </c>
-      <c r="M24" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="N24" s="10" t="s">
-        <v>12</v>
+      <c r="K24" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L24" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M24" s="6">
+        <v>20</v>
+      </c>
+      <c r="N24" s="6">
+        <v>1</v>
       </c>
       <c r="O24" s="10" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="25" spans="1:20">
+      <c r="P24" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q24" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22">
       <c r="A25" s="6" t="s">
         <v>64</v>
       </c>
@@ -2061,23 +2207,29 @@
       <c r="J25" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K25" s="6">
-        <v>20</v>
-      </c>
-      <c r="L25" s="6">
+      <c r="K25" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L25" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="M25" s="6">
+        <v>20</v>
+      </c>
+      <c r="N25" s="6">
         <v>3</v>
       </c>
-      <c r="M25" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N25" s="10" t="s">
-        <v>12</v>
-      </c>
       <c r="O25" s="10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="26" spans="1:20">
+        <v>12</v>
+      </c>
+      <c r="P25" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q25" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22">
       <c r="A26" s="6" t="s">
         <v>65</v>
       </c>
@@ -2108,29 +2260,35 @@
       <c r="J26" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K26" s="6">
-        <v>20</v>
-      </c>
-      <c r="L26" s="6">
+      <c r="K26" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="L26" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M26" s="6">
+        <v>20</v>
+      </c>
+      <c r="N26" s="6">
         <v>2</v>
       </c>
-      <c r="M26" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N26" s="10" t="s">
-        <v>12</v>
-      </c>
       <c r="O26" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="S26" t="s">
+        <v>12</v>
+      </c>
+      <c r="P26" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q26" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="U26" t="s">
         <v>66</v>
       </c>
-      <c r="T26" t="s">
+      <c r="V26" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="27" spans="1:20">
+    <row r="27" spans="1:22">
       <c r="A27" s="6" t="s">
         <v>68</v>
       </c>
@@ -2161,32 +2319,38 @@
       <c r="J27" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K27" s="6">
-        <v>20</v>
-      </c>
-      <c r="L27" s="6">
-        <v>1</v>
-      </c>
-      <c r="M27" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N27" s="10" t="s">
-        <v>12</v>
+      <c r="K27" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L27" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M27" s="6">
+        <v>20</v>
+      </c>
+      <c r="N27" s="6">
+        <v>1</v>
       </c>
       <c r="O27" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="R27" s="5" t="s">
+      <c r="P27" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q27" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="T27" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="S27">
+      <c r="U27">
         <v>8</v>
       </c>
-      <c r="T27">
+      <c r="V27">
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:20">
+    <row r="28" spans="1:22">
       <c r="A28" s="6" t="s">
         <v>70</v>
       </c>
@@ -2215,30 +2379,36 @@
       <c r="J28" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K28" s="6">
+      <c r="K28" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L28" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M28" s="6">
         <v>0</v>
       </c>
-      <c r="L28" s="6"/>
-      <c r="M28" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="N28" s="6" t="s">
-        <v>11</v>
-      </c>
+      <c r="N28" s="6"/>
       <c r="O28" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="R28" s="5" t="s">
+      <c r="P28" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q28" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="T28" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="S28">
+      <c r="U28">
         <v>8</v>
       </c>
-      <c r="T28">
+      <c r="V28">
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:20">
+    <row r="29" spans="1:22">
       <c r="A29" s="6" t="s">
         <v>72</v>
       </c>
@@ -2269,23 +2439,29 @@
       <c r="J29" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K29" s="6">
-        <v>20</v>
-      </c>
-      <c r="L29" s="6">
+      <c r="K29" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L29" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M29" s="6">
+        <v>20</v>
+      </c>
+      <c r="N29" s="6">
         <v>2</v>
       </c>
-      <c r="M29" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N29" s="10" t="s">
-        <v>12</v>
-      </c>
       <c r="O29" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="30" spans="1:20">
+      <c r="P29" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q29" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22">
       <c r="A30" s="6" t="s">
         <v>73</v>
       </c>
@@ -2316,23 +2492,29 @@
       <c r="J30" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K30" s="6">
-        <v>20</v>
-      </c>
-      <c r="L30" s="6">
-        <v>1</v>
-      </c>
-      <c r="M30" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N30" s="10" t="s">
-        <v>12</v>
+      <c r="K30" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L30" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M30" s="6">
+        <v>20</v>
+      </c>
+      <c r="N30" s="6">
+        <v>1</v>
       </c>
       <c r="O30" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="31" spans="1:20">
+      <c r="P30" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q30" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22">
       <c r="A31" s="6" t="s">
         <v>74</v>
       </c>
@@ -2363,23 +2545,29 @@
       <c r="J31" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K31" s="6">
-        <v>20</v>
-      </c>
-      <c r="L31" s="6">
+      <c r="K31" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L31" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M31" s="6">
+        <v>20</v>
+      </c>
+      <c r="N31" s="6">
         <v>2</v>
       </c>
-      <c r="M31" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N31" s="10" t="s">
-        <v>12</v>
-      </c>
       <c r="O31" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="32" spans="1:20">
+      <c r="P31" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q31" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32" spans="1:22">
       <c r="A32" s="6" t="s">
         <v>75</v>
       </c>
@@ -2410,23 +2598,29 @@
       <c r="J32" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K32" s="6">
-        <v>20</v>
-      </c>
-      <c r="L32" s="6">
+      <c r="K32" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L32" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M32" s="6">
+        <v>20</v>
+      </c>
+      <c r="N32" s="6">
         <v>2</v>
       </c>
-      <c r="M32" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N32" s="10" t="s">
-        <v>12</v>
-      </c>
       <c r="O32" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="33" spans="1:15">
+      <c r="P32" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q32" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17">
       <c r="A33" s="6" t="s">
         <v>76</v>
       </c>
@@ -2457,23 +2651,29 @@
       <c r="J33" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K33" s="6">
-        <v>20</v>
-      </c>
-      <c r="L33" s="6">
-        <v>1</v>
-      </c>
-      <c r="M33" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N33" s="10" t="s">
-        <v>12</v>
+      <c r="K33" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L33" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M33" s="6">
+        <v>20</v>
+      </c>
+      <c r="N33" s="6">
+        <v>1</v>
       </c>
       <c r="O33" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="34" spans="1:15">
+      <c r="P33" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q33" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17">
       <c r="A34" s="11" t="s">
         <v>77</v>
       </c>
@@ -2504,23 +2704,29 @@
       <c r="J34" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K34" s="11">
-        <v>20</v>
-      </c>
-      <c r="L34" s="11">
-        <v>1</v>
-      </c>
-      <c r="M34" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N34" s="10" t="s">
-        <v>12</v>
+      <c r="K34" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L34" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M34" s="11">
+        <v>20</v>
+      </c>
+      <c r="N34" s="11">
+        <v>1</v>
       </c>
       <c r="O34" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="35" spans="1:15">
+      <c r="P34" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q34" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17">
       <c r="A35" s="6" t="s">
         <v>78</v>
       </c>
@@ -2551,23 +2757,29 @@
       <c r="J35" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="K35" s="6">
-        <v>20</v>
-      </c>
-      <c r="L35" s="6">
+      <c r="K35" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L35" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M35" s="6">
+        <v>20</v>
+      </c>
+      <c r="N35" s="6">
         <v>4</v>
       </c>
-      <c r="M35" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N35" s="10" t="s">
-        <v>12</v>
-      </c>
       <c r="O35" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="36" spans="1:15">
+      <c r="P35" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q35" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17">
       <c r="A36" s="6" t="s">
         <v>79</v>
       </c>
@@ -2596,21 +2808,27 @@
       <c r="J36" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K36" s="6">
+      <c r="K36" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L36" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M36" s="6">
         <v>0</v>
       </c>
-      <c r="L36" s="6"/>
-      <c r="M36" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="N36" s="6" t="s">
-        <v>11</v>
-      </c>
+      <c r="N36" s="6"/>
       <c r="O36" s="6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="37" spans="1:15">
+      <c r="P36" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q36" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17">
       <c r="A37" s="6" t="s">
         <v>80</v>
       </c>
@@ -2639,23 +2857,29 @@
       <c r="J37" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K37" s="6">
-        <v>20</v>
-      </c>
-      <c r="L37" s="6">
-        <v>1</v>
-      </c>
-      <c r="M37" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N37" s="10" t="s">
-        <v>12</v>
+      <c r="K37" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L37" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M37" s="6">
+        <v>20</v>
+      </c>
+      <c r="N37" s="6">
+        <v>1</v>
       </c>
       <c r="O37" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="38" spans="1:15">
+      <c r="P37" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q37" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17">
       <c r="A38" s="6" t="s">
         <v>81</v>
       </c>
@@ -2684,23 +2908,29 @@
       <c r="J38" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K38" s="6">
-        <v>20</v>
-      </c>
-      <c r="L38" s="6">
-        <v>1</v>
-      </c>
-      <c r="M38" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N38" s="10" t="s">
-        <v>12</v>
+      <c r="K38" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L38" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M38" s="6">
+        <v>20</v>
+      </c>
+      <c r="N38" s="6">
+        <v>1</v>
       </c>
       <c r="O38" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="39" spans="1:15">
+      <c r="P38" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q38" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17">
       <c r="A39" s="6" t="s">
         <v>82</v>
       </c>
@@ -2729,23 +2959,29 @@
       <c r="J39" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K39" s="6">
-        <v>20</v>
-      </c>
-      <c r="L39" s="6">
-        <v>1</v>
-      </c>
-      <c r="M39" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N39" s="10" t="s">
-        <v>12</v>
+      <c r="K39" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L39" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M39" s="6">
+        <v>20</v>
+      </c>
+      <c r="N39" s="6">
+        <v>1</v>
       </c>
       <c r="O39" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="40" spans="1:15">
+      <c r="P39" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q39" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17">
       <c r="A40" s="6" t="s">
         <v>83</v>
       </c>
@@ -2774,23 +3010,29 @@
       <c r="J40" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K40" s="6">
-        <v>20</v>
-      </c>
-      <c r="L40" s="6">
-        <v>1</v>
-      </c>
-      <c r="M40" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N40" s="10" t="s">
-        <v>12</v>
+      <c r="K40" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L40" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M40" s="6">
+        <v>20</v>
+      </c>
+      <c r="N40" s="6">
+        <v>1</v>
       </c>
       <c r="O40" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="41" spans="1:15">
+      <c r="P40" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q40" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17">
       <c r="A41" s="6" t="s">
         <v>84</v>
       </c>
@@ -2819,23 +3061,29 @@
       <c r="J41" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K41" s="6">
-        <v>20</v>
-      </c>
-      <c r="L41" s="6">
-        <v>1</v>
-      </c>
-      <c r="M41" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N41" s="10" t="s">
-        <v>12</v>
+      <c r="K41" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L41" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M41" s="6">
+        <v>20</v>
+      </c>
+      <c r="N41" s="6">
+        <v>1</v>
       </c>
       <c r="O41" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="42" spans="1:15">
+      <c r="P41" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q41" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17">
       <c r="A42" s="6" t="s">
         <v>85</v>
       </c>
@@ -2864,23 +3112,29 @@
       <c r="J42" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K42" s="6">
-        <v>20</v>
-      </c>
-      <c r="L42" s="6">
-        <v>1</v>
-      </c>
-      <c r="M42" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N42" s="10" t="s">
-        <v>12</v>
+      <c r="K42" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L42" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M42" s="6">
+        <v>20</v>
+      </c>
+      <c r="N42" s="6">
+        <v>1</v>
       </c>
       <c r="O42" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="43" spans="1:15">
+      <c r="P42" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q42" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17">
       <c r="A43" s="9" t="s">
         <v>86</v>
       </c>
@@ -2909,23 +3163,29 @@
       <c r="J43" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K43" s="6">
+      <c r="K43" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L43" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M43" s="6">
         <v>80</v>
       </c>
-      <c r="L43" s="6">
+      <c r="N43" s="6">
         <v>2</v>
       </c>
-      <c r="M43" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="N43" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="O43" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="44" spans="1:15">
+      <c r="O43" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="P43" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q43" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17">
       <c r="A44" s="12" t="s">
         <v>87</v>
       </c>
@@ -2956,23 +3216,29 @@
       <c r="J44" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K44" s="6">
-        <v>20</v>
-      </c>
-      <c r="L44" s="6">
-        <v>1</v>
-      </c>
-      <c r="M44" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N44" s="10" t="s">
-        <v>12</v>
+      <c r="K44" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L44" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M44" s="6">
+        <v>20</v>
+      </c>
+      <c r="N44" s="6">
+        <v>1</v>
       </c>
       <c r="O44" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="45" spans="1:15">
+      <c r="P44" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q44" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="45" spans="1:17">
       <c r="A45" s="6" t="s">
         <v>88</v>
       </c>
@@ -3001,23 +3267,29 @@
       <c r="J45" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K45" s="6">
-        <v>20</v>
-      </c>
-      <c r="L45" s="6">
-        <v>1</v>
-      </c>
-      <c r="M45" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N45" s="10" t="s">
-        <v>12</v>
+      <c r="K45" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L45" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M45" s="6">
+        <v>20</v>
+      </c>
+      <c r="N45" s="6">
+        <v>1</v>
       </c>
       <c r="O45" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="46" spans="1:15">
+      <c r="P45" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q45" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17">
       <c r="A46" s="6" t="s">
         <v>89</v>
       </c>
@@ -3046,23 +3318,29 @@
       <c r="J46" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K46" s="6">
-        <v>20</v>
-      </c>
-      <c r="L46" s="6">
-        <v>1</v>
-      </c>
-      <c r="M46" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N46" s="10" t="s">
-        <v>12</v>
+      <c r="K46" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L46" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M46" s="6">
+        <v>20</v>
+      </c>
+      <c r="N46" s="6">
+        <v>1</v>
       </c>
       <c r="O46" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="47" spans="1:15">
+      <c r="P46" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q46" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17">
       <c r="A47" s="9" t="s">
         <v>90</v>
       </c>
@@ -3093,23 +3371,29 @@
       <c r="J47" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K47" s="6">
-        <v>20</v>
-      </c>
-      <c r="L47" s="6">
-        <v>1</v>
-      </c>
-      <c r="M47" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N47" s="10" t="s">
-        <v>12</v>
+      <c r="K47" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L47" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M47" s="6">
+        <v>20</v>
+      </c>
+      <c r="N47" s="6">
+        <v>1</v>
       </c>
       <c r="O47" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="48" spans="1:15">
+      <c r="P47" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q47" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="48" spans="1:17">
       <c r="A48" s="6" t="s">
         <v>91</v>
       </c>
@@ -3140,19 +3424,25 @@
       <c r="J48" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K48" s="6">
-        <v>20</v>
-      </c>
-      <c r="L48" s="6">
-        <v>1</v>
-      </c>
-      <c r="M48" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="N48" s="10" t="s">
-        <v>12</v>
+      <c r="K48" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L48" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="M48" s="6">
+        <v>20</v>
+      </c>
+      <c r="N48" s="6">
+        <v>1</v>
       </c>
       <c r="O48" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="P48" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q48" s="10" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>